<commit_message>
feat: new excel file model, tirage live added + a btn toggle for each option, temporary css for tests
</commit_message>
<xml_diff>
--- a/assets/modele-participants.xlsx
+++ b/assets/modele-participants.xlsx
@@ -451,12 +451,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -470,11 +469,6 @@
           <t>Email</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Exclusion</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -487,7 +481,6 @@
           <t>camille@email.com</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -500,11 +493,6 @@
           <t>yanis@email.com</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Camille</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -517,57 +505,46 @@
           <t>lina@email.com</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="n"/>
       <c r="B5" s="3" t="n"/>
-      <c r="C5" s="3" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="n"/>
       <c r="B6" s="3" t="n"/>
-      <c r="C6" s="3" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="3" t="n"/>
       <c r="B7" s="3" t="n"/>
-      <c r="C7" s="3" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="n"/>
       <c r="B8" s="3" t="n"/>
-      <c r="C8" s="3" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="3" t="n"/>
       <c r="B9" s="3" t="n"/>
-      <c r="C9" s="3" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="3" t="n"/>
       <c r="B10" s="3" t="n"/>
-      <c r="C10" s="3" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="3" t="n"/>
       <c r="B11" s="3" t="n"/>
-      <c r="C11" s="3" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="3" t="n"/>
       <c r="B12" s="3" t="n"/>
-      <c r="C12" s="3" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="3" t="n"/>
       <c r="B13" s="3" t="n"/>
-      <c r="C13" s="3" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="3" t="n"/>
       <c r="B14" s="3" t="n"/>
-      <c r="C14" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -599,7 +576,7 @@
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>1. Ne modifiez pas les noms des colonnes (Prénom, Email, Exclusion) dans l'onglet "Participants".</t>
+          <t>1. Ne modifiez pas les noms des colonnes (Prénom, Email) dans l'onglet "Participants".</t>
         </is>
       </c>
     </row>
@@ -613,21 +590,21 @@
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>3. La colonne "Exclusion" est facultative : indiquez le prénom exact d'une personne que ce participant ne doit pas tirer au sort (ex. son conjoint).</t>
+          <t>3. Les trois premières lignes de l'onglet "Participants" sont des exemples en italique — vous pouvez les remplacer ou les supprimer.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>4. Les trois premières lignes de l'onglet "Participants" sont des exemples en italique — vous pouvez les remplacer ou les supprimer.</t>
+          <t>4. Une fois complété, importez ce fichier depuis le site pour remplir automatiquement le formulaire.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>5. Une fois complété, importez ce fichier depuis le site pour remplir automatiquement le formulaire.</t>
+          <t>5. Les exclusions (personnes à ne pas associer entre elles) se définissent ensuite directement sur le site, après l'import.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: nav modified, new pages created, generic css for non-index pages, new excel asset,  fix minors details
</commit_message>
<xml_diff>
--- a/assets/modele-participants.xlsx
+++ b/assets/modele-participants.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -30,25 +30,15 @@
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <i val="1"/>
-      <color rgb="00808080"/>
-    </font>
-    <font>
-      <name val="Arial"/>
     </font>
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="001B3A2F"/>
-      <sz val="13"/>
+      <sz val="12"/>
     </font>
     <font>
       <name val="Arial"/>
-      <sz val="11"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="3">
@@ -61,7 +51,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001B3A2F"/>
-        <bgColor rgb="001B3A2F"/>
       </patternFill>
     </fill>
   </fills>
@@ -77,15 +66,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -451,11 +440,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -471,80 +460,40 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>Camille</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>camille@email.com</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>Yanis</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>yanis@email.com</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>Lina</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>lina@email.com</t>
         </is>
       </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="3" t="n"/>
-      <c r="B5" s="3" t="n"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="3" t="n"/>
-      <c r="B6" s="3" t="n"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="3" t="n"/>
-      <c r="B7" s="3" t="n"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="3" t="n"/>
-      <c r="B8" s="3" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="3" t="n"/>
-      <c r="B9" s="3" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="3" t="n"/>
-      <c r="B10" s="3" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="n"/>
-      <c r="B11" s="3" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="3" t="n"/>
-      <c r="B12" s="3" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="n"/>
-      <c r="B13" s="3" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="n"/>
-      <c r="B14" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -557,54 +506,91 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A7"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="90" customWidth="1" min="1" max="1"/>
+    <col width="100" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>Comment remplir ce fichier</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="inlineStr"/>
+      <c r="A2" s="3" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>1. Ne modifiez pas les noms des colonnes (Prénom, Email) dans l'onglet "Participants".</t>
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>1. Gardez la ligne d'en-tête telle quelle : Prénom | Email (ne changez pas l'orthographe).</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="inlineStr">
-        <is>
-          <t>2. Une ligne = un participant.</t>
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>2. Une ligne = un participant (3 minimum, 50 maximum).</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="inlineStr">
-        <is>
-          <t>3. Les trois premières lignes de l'onglet "Participants" sont des exemples en italique — vous pouvez les remplacer ou les supprimer.</t>
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>3. Les prénoms doivent être uniques (ex. Marie L. et Marie D.).</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>4. Une fois complété, importez ce fichier depuis le site pour remplir automatiquement le formulaire.</t>
-        </is>
-      </c>
+      <c r="A6" s="3" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>5. Les exclusions (personnes à ne pas associer entre elles) se définissent ensuite directement sur le site, après l'import.</t>
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Tirage par e-mail</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Prénom et Email sont obligatoires. Une ligne sans email est ignorée.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Tirage « live »</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Seule la colonne Prénom est utilisée. La colonne Email est ignorée : vous pouvez la laisser vide ou la supprimer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Les exclusions se règlent directement sur le site, après l'import.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Ne modifiez pas le nom de la feuille « Participants » (le site lit la première feuille du fichier).</t>
         </is>
       </c>
     </row>

</xml_diff>